<commit_message>
ACTUALIZACION PLANILLA DE EV
</commit_message>
<xml_diff>
--- a/Fase 1/Evidencias Grupales/PLANILLA DE EVALUACIÓN FASE 1.xlsx
+++ b/Fase 1/Evidencias Grupales/PLANILLA DE EVALUACIÓN FASE 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6a0a8af1cc48dbc0/2025-2/CAPSTONE/Documentos_por_fase/DOCUMENTOS FASE1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\duoc\SM2-2026\Capstone-PTY4614-001V\Grupos\Grupo 12 Cosmelli\Fase 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="612" documentId="8_{2EFDF332-31E9-4C74-A6B5-E695634C1C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15C90F07-E4D5-4EBF-AE4C-FB79430617FF}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00ED87B7-1000-461E-8297-EE958A09A7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="98">
   <si>
     <t>INTEGRANTES</t>
   </si>
@@ -379,6 +379,15 @@
   <si>
     <t>Muy Relevante</t>
   </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Francisco Cosmelli</t>
+  </si>
 </sst>
 </file>
 
@@ -477,7 +486,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -523,6 +532,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF262626"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -907,7 +922,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1039,6 +1054,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -1439,7 +1460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:K929"/>
+  <dimension ref="A2:K927"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -1461,9 +1482,10 @@
       <c r="D2" s="2">
         <v>0.25</v>
       </c>
-      <c r="E2" s="63">
+      <c r="E2" s="65">
         <v>1</v>
       </c>
+      <c r="G2" s="49"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
@@ -1475,672 +1497,701 @@
       <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="50"/>
+      <c r="E3" s="52"/>
+      <c r="G3" s="49"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>1</v>
       </c>
-      <c r="B4" s="32"/>
+      <c r="B4" s="32" t="s">
+        <v>97</v>
+      </c>
       <c r="C4" s="6">
-        <f>EVALUACION1!$C$24</f>
+        <f>EVALUACION1!$C$22</f>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="D4" s="6">
+        <f>$C$33</f>
+        <v>6</v>
+      </c>
+      <c r="E4" s="43">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="G4" s="49"/>
+    </row>
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G5" s="49"/>
+    </row>
+    <row r="9" spans="1:11" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="66" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="14"/>
+      <c r="C9" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="E9" s="64"/>
+      <c r="F9" s="64"/>
+      <c r="G9" s="64"/>
+      <c r="H9" s="64"/>
+      <c r="I9" s="64"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="61"/>
+    </row>
+    <row r="10" spans="1:11" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="63"/>
+      <c r="B10" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="52"/>
+      <c r="D10" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="6">
-        <f>$C$35</f>
-        <v>7</v>
-      </c>
-      <c r="E4" s="43">
-        <f>C4*C$2+D4*D$2</f>
-        <v>7</v>
-      </c>
-      <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
-        <v>2</v>
-      </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="6">
-        <f>EVALUACION1!$C$24</f>
-        <v>7</v>
-      </c>
-      <c r="D5" s="6">
-        <f>C47</f>
-        <v>7</v>
-      </c>
-      <c r="E5" s="43">
-        <f t="shared" ref="E5:E6" si="0">C5*C$2+D5*D$2</f>
-        <v>7</v>
-      </c>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="5">
-        <v>3</v>
-      </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="6">
-        <f>EVALUACION1!$C$24</f>
-        <v>7</v>
-      </c>
-      <c r="D6" s="6">
-        <f>C58</f>
-        <v>7</v>
-      </c>
-      <c r="E6" s="43">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="11" spans="1:11" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="64" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="51" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="58" t="s">
-        <v>5</v>
-      </c>
-      <c r="E11" s="62"/>
-      <c r="F11" s="62"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
-      <c r="I11" s="62"/>
-      <c r="J11" s="62"/>
-      <c r="K11" s="59"/>
-    </row>
-    <row r="12" spans="1:11" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="61"/>
-      <c r="B12" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="50"/>
-      <c r="D12" s="58" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="59"/>
-      <c r="F12" s="58" t="s">
+      <c r="E10" s="61"/>
+      <c r="F10" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="G12" s="59"/>
-      <c r="H12" s="58" t="s">
+      <c r="G10" s="61"/>
+      <c r="H10" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="I12" s="59"/>
-      <c r="J12" s="58" t="s">
+      <c r="I10" s="61"/>
+      <c r="J10" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="K12" s="59"/>
-    </row>
-    <row r="13" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="65"/>
-      <c r="B13" s="35" t="str">
+      <c r="K10" s="61"/>
+    </row>
+    <row r="11" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="67"/>
+      <c r="B11" s="35" t="str">
         <f>RUBRICA!A5</f>
         <v>1. Describe brevemente en qué consiste el Proyecto APT, justificando su relevancia para el campo laboral de su carrera.</v>
       </c>
+      <c r="C11" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="16">
+        <f>IF(D11="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F11" s="16" t="str">
+        <f t="shared" ref="F11:F12" si="0">IF($C11=L,"X","")</f>
+        <v/>
+      </c>
+      <c r="G11" s="16" t="str">
+        <f>IF(F11="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="16" t="str">
+        <f t="shared" ref="H11:H14" si="1">IF($C11=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I11" s="16" t="str">
+        <f>IF(H11="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="16" t="str">
+        <f t="shared" ref="J11:J14" si="2">IF($C11=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K11" s="16" t="str">
+        <f t="shared" ref="K11:K14" si="3">IF($J11="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="26.45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="67"/>
+      <c r="B12" s="35" t="str">
+        <f>RUBRICA!A6</f>
+        <v>2. Relaciona el Proyecto APT con las competencias del perfil de egreso de su Plan de Estudio.</v>
+      </c>
+      <c r="C12" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E12" s="16">
+        <f t="shared" ref="E12" si="4">IF(D12="X",100*0.05,"")</f>
+        <v>5</v>
+      </c>
+      <c r="F12" s="16" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G12" s="16" t="str">
+        <f t="shared" ref="G12" si="5">IF(F12="X",60*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I12" s="16" t="str">
+        <f t="shared" ref="I12" si="6">IF(H12="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="K12" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="67"/>
+      <c r="B13" s="35" t="str">
+        <f>RUBRICA!A8</f>
+        <v xml:space="preserve">4.  Argumenta por qué el proyecto es factible de realizarse en el marco de la asignatura. </v>
+      </c>
       <c r="C13" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="16" t="str">
-        <f t="shared" ref="D13:D16" si="1">IF($C13=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E13" s="16">
-        <f>IF(D13="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F13" s="16" t="str">
-        <f t="shared" ref="F13:F16" si="2">IF($C13=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G13" s="16" t="str">
-        <f>IF(F13="X",60*0.1,"")</f>
-        <v/>
+      <c r="D13" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E13" s="16" t="str">
+        <f t="shared" ref="E13:E19" si="7">IF(D13="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="16">
+        <f t="shared" ref="G13:G19" si="8">IF(F13="X",60*0.05,"")</f>
+        <v>3</v>
       </c>
       <c r="H13" s="16" t="str">
-        <f t="shared" ref="H13:H16" si="3">IF($C13=ML,"X","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="I13" s="16" t="str">
-        <f>IF(H13="X",30*0.1,"")</f>
+        <f t="shared" ref="I13:I19" si="9">IF(H13="X",30*0.05,"")</f>
         <v/>
       </c>
       <c r="J13" s="16" t="str">
-        <f t="shared" ref="J13:J16" si="4">IF($C13=NL,"X","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="K13" s="16" t="str">
-        <f t="shared" ref="K13:K16" si="5">IF($J13="X",0,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="26.45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="65"/>
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="67"/>
       <c r="B14" s="35" t="str">
-        <f>RUBRICA!A6</f>
-        <v>2. Relaciona el Proyecto APT con las competencias del perfil de egreso de su Plan de Estudio.</v>
+        <f>RUBRICA!A9</f>
+        <v xml:space="preserve">5. Formula objetivos claros, concisos y coherentes con la disciplina y la situación a abordar. </v>
       </c>
       <c r="C14" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D14" s="16" t="str">
+      <c r="D14" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E14" s="16" t="str">
+        <f>IF(D14="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" s="16">
+        <f>IF(F14="X",60*0.05,"")</f>
+        <v>3</v>
+      </c>
+      <c r="H14" s="16" t="str">
         <f t="shared" si="1"/>
-        <v>X</v>
-      </c>
-      <c r="E14" s="16">
-        <f t="shared" ref="E14" si="6">IF(D14="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F14" s="16" t="str">
+        <v/>
+      </c>
+      <c r="I14" s="16" t="str">
+        <f>IF(H14="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="16" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="G14" s="16" t="str">
-        <f t="shared" ref="G14" si="7">IF(F14="X",60*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="16" t="str">
+      <c r="K14" s="16" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="I14" s="16" t="str">
-        <f t="shared" ref="I14" si="8">IF(H14="X",30*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="16" t="str">
-        <f t="shared" si="4"/>
-        <v/>
-      </c>
-      <c r="K14" s="16" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
     </row>
     <row r="15" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="65"/>
+      <c r="A15" s="67"/>
       <c r="B15" s="35" t="str">
-        <f>RUBRICA!A8</f>
-        <v xml:space="preserve">4.  Argumenta por qué el proyecto es factible de realizarse en el marco de la asignatura. </v>
+        <f>RUBRICA!A10</f>
+        <v>6. Propone una metodología de trabajo que permite alcanzar los objetivos propuestos y es pertinente con los requerimientos disciplinares.</v>
       </c>
       <c r="C15" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="16" t="str">
-        <f t="shared" si="1"/>
-        <v>X</v>
-      </c>
-      <c r="E15" s="16">
-        <f t="shared" ref="E15:E21" si="9">IF(D15="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F15" s="16" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="G15" s="16" t="str">
-        <f t="shared" ref="G15:G21" si="10">IF(F15="X",60*0.05,"")</f>
-        <v/>
+      <c r="D15" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E15" s="16" t="str">
+        <f t="shared" ref="E15" si="10">IF(D15="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" s="16">
+        <f t="shared" ref="G15" si="11">IF(F15="X",60*0.1,"")</f>
+        <v>6</v>
       </c>
       <c r="H15" s="16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="H15:H20" si="12">IF($C15=ML,"X","")</f>
         <v/>
       </c>
       <c r="I15" s="16" t="str">
-        <f t="shared" ref="I15:I21" si="11">IF(H15="X",30*0.05,"")</f>
+        <f t="shared" ref="I15" si="13">IF(H15="X",30*0.1,"")</f>
         <v/>
       </c>
       <c r="J15" s="16" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="J15:J20" si="14">IF($C15=NL,"X","")</f>
         <v/>
       </c>
       <c r="K15" s="16" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="K15:K20" si="15">IF($J15="X",0,"")</f>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="65"/>
+      <c r="A16" s="67"/>
       <c r="B16" s="35" t="str">
-        <f>RUBRICA!A9</f>
-        <v xml:space="preserve">5. Formula objetivos claros, concisos y coherentes con la disciplina y la situación a abordar. </v>
+        <f>RUBRICA!A11</f>
+        <v xml:space="preserve">7. Establece un plan de trabajo para su proyecto APT considerando los recursos, duración, facilitadores y obstaculizadores en el desarrollo de las actividades. </v>
       </c>
       <c r="C16" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D16" s="16" t="str">
-        <f t="shared" si="1"/>
-        <v>X</v>
-      </c>
-      <c r="E16" s="16">
-        <f>IF(D16="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F16" s="16" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="G16" s="16" t="str">
-        <f>IF(F16="X",60*0.05,"")</f>
-        <v/>
+      <c r="D16" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E16" s="16" t="str">
+        <f t="shared" ref="E16" si="16">IF(D16="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G16" s="16">
+        <f t="shared" ref="G16" si="17">IF(F16="X",60*0.1,"")</f>
+        <v>6</v>
       </c>
       <c r="H16" s="16" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="I16" s="16" t="str">
-        <f>IF(H16="X",30*0.05,"")</f>
+        <f t="shared" ref="I16" si="18">IF(H16="X",30*0.1,"")</f>
         <v/>
       </c>
       <c r="J16" s="16" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="K16" s="16" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
     </row>
     <row r="17" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="65"/>
+      <c r="A17" s="67"/>
       <c r="B17" s="35" t="str">
-        <f>RUBRICA!A10</f>
-        <v>6. Propone una metodología de trabajo que permite alcanzar los objetivos propuestos y es pertinente con los requerimientos disciplinares.</v>
+        <f>RUBRICA!A12</f>
+        <v>8. Determina evidencias, justificando cómo estas dan cuenta del logro de las actividades del Proyecto APT.</v>
       </c>
       <c r="C17" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="16" t="str">
-        <f t="shared" ref="D17:D22" si="12">IF($C17=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E17" s="16">
-        <f t="shared" ref="E17" si="13">IF(D17="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F17" s="16" t="str">
-        <f t="shared" ref="F17:F22" si="14">IF($C17=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G17" s="16" t="str">
-        <f t="shared" ref="G17" si="15">IF(F17="X",60*0.1,"")</f>
-        <v/>
+      <c r="D17" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E17" s="16" t="str">
+        <f>IF(D17="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F17" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" s="16">
+        <f t="shared" ref="G17" si="19">IF(F17="X",60*0.05,"")</f>
+        <v>3</v>
       </c>
       <c r="H17" s="16" t="str">
-        <f t="shared" ref="H17:H22" si="16">IF($C17=ML,"X","")</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="I17" s="16" t="str">
-        <f t="shared" ref="I17" si="17">IF(H17="X",30*0.1,"")</f>
+        <f t="shared" ref="I17" si="20">IF(H17="X",30*0.05,"")</f>
         <v/>
       </c>
       <c r="J17" s="16" t="str">
-        <f t="shared" ref="J17:J22" si="18">IF($C17=NL,"X","")</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
       <c r="K17" s="16" t="str">
-        <f t="shared" ref="K17:K22" si="19">IF($J17="X",0,"")</f>
+        <f t="shared" si="15"/>
         <v/>
       </c>
     </row>
     <row r="18" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="65"/>
-      <c r="B18" s="35" t="str">
-        <f>RUBRICA!A11</f>
-        <v xml:space="preserve">7. Establece un plan de trabajo para su proyecto APT considerando los recursos, duración, facilitadores y obstaculizadores en el desarrollo de las actividades. </v>
+      <c r="A18" s="67"/>
+      <c r="B18" s="50" t="str">
+        <f>RUBRICA!A13</f>
+        <v xml:space="preserve">9. Utiliza reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </v>
       </c>
       <c r="C18" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="16" t="str">
+      <c r="D18" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="16" t="str">
+        <f>IF(D18="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G18" s="16">
+        <f t="shared" si="8"/>
+        <v>3</v>
+      </c>
+      <c r="H18" s="16" t="str">
         <f t="shared" si="12"/>
-        <v>X</v>
-      </c>
-      <c r="E18" s="16">
-        <f t="shared" ref="E18" si="20">IF(D18="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F18" s="16" t="str">
+        <v/>
+      </c>
+      <c r="I18" s="16" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="J18" s="16" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="G18" s="16" t="str">
-        <f t="shared" ref="G18" si="21">IF(F18="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="16" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="I18" s="16" t="str">
-        <f t="shared" ref="I18" si="22">IF(H18="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
       <c r="K18" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="65"/>
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="22.9" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="67"/>
       <c r="B19" s="35" t="str">
-        <f>RUBRICA!A12</f>
-        <v>8. Determina evidencias, justificando cómo estas dan cuenta del logro de las actividades del Proyecto APT.</v>
+        <f>RUBRICA!A14</f>
+        <v>10. Cumple completando el contenido del informe de presentación del proyecto de acuerdo con la plantilla entregada.</v>
       </c>
       <c r="C19" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="16" t="str">
+      <c r="D19" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="F19" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G19" s="16">
+        <f t="shared" si="8"/>
+        <v>3</v>
+      </c>
+      <c r="H19" s="16" t="str">
         <f t="shared" si="12"/>
-        <v>X</v>
-      </c>
-      <c r="E19" s="16">
-        <f>IF(D19="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F19" s="16" t="str">
+        <v/>
+      </c>
+      <c r="I19" s="16" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+      <c r="J19" s="16" t="str">
         <f t="shared" si="14"/>
         <v/>
       </c>
-      <c r="G19" s="16" t="str">
-        <f t="shared" ref="G19" si="23">IF(F19="X",60*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="H19" s="16" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="I19" s="16" t="str">
-        <f t="shared" ref="I19" si="24">IF(H19="X",30*0.05,"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
       <c r="K19" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="65"/>
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="36" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="67"/>
       <c r="B20" s="35" t="str">
-        <f>RUBRICA!A13</f>
-        <v xml:space="preserve">9. Utiliza reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </v>
-      </c>
-      <c r="C20" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="16" t="str">
-        <f t="shared" si="12"/>
-        <v>X</v>
-      </c>
-      <c r="E20" s="16">
-        <f>IF(D20="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F20" s="16" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="G20" s="16" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="H20" s="16" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="I20" s="16" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="J20" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="K20" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="22.9" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="65"/>
-      <c r="B21" s="35" t="str">
-        <f>RUBRICA!A14</f>
-        <v>10. Cumple completando el contenido del informe de presentación del proyecto de acuerdo con la plantilla entregada.</v>
-      </c>
-      <c r="C21" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="16" t="str">
-        <f t="shared" si="12"/>
-        <v>X</v>
-      </c>
-      <c r="E21" s="16">
-        <f t="shared" si="9"/>
-        <v>5</v>
-      </c>
-      <c r="F21" s="16" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="G21" s="16" t="str">
-        <f t="shared" si="10"/>
-        <v/>
-      </c>
-      <c r="H21" s="16" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="I21" s="16" t="str">
-        <f t="shared" si="11"/>
-        <v/>
-      </c>
-      <c r="J21" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="K21" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="36" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="65"/>
-      <c r="B22" s="35" t="str">
         <f>RUBRICA!A16</f>
         <v>12. Desarrolla un plan de trabajo que permita del logro de los objetivos propuestos del proyecto de 
 acuerdo a los tiempos para su desarrollo</v>
       </c>
-      <c r="C22" s="33" t="s">
+      <c r="C20" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="16" t="str">
+      <c r="D20" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E20" s="16" t="str">
+        <f>IF(D20="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G20" s="16">
+        <f>IF(F20="X",60*0.1,"")</f>
+        <v>6</v>
+      </c>
+      <c r="H20" s="16" t="str">
         <f t="shared" si="12"/>
-        <v>X</v>
-      </c>
-      <c r="E22" s="16">
-        <f>IF(D22="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="I20" s="16" t="str">
+        <f>IF(H20="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+      <c r="K20" s="16" t="str">
+        <f t="shared" si="15"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="63"/>
+      <c r="B21" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="37">
+        <f>E21+G21+I21+K21</f>
+        <v>48</v>
+      </c>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19">
+        <f>SUM(E11:E20)</f>
+        <v>15</v>
+      </c>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19">
+        <f>SUM(G11:G20)</f>
+        <v>33</v>
+      </c>
+      <c r="H21" s="19"/>
+      <c r="I21" s="19">
+        <f>SUM(I11:I20)</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19">
+        <f>SUM(K11:K20)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="52"/>
+      <c r="B22" s="36" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="20">
+        <f>VLOOKUP(C21,ESCALA_IEP!A2:B142,2,FALSE)</f>
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="54" t="str">
+        <f>$B$4</f>
+        <v>Francisco Cosmelli</v>
+      </c>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="55"/>
+      <c r="J25" s="55"/>
+      <c r="K25" s="56"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="63"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+      <c r="F26" s="58"/>
+      <c r="G26" s="58"/>
+      <c r="H26" s="58"/>
+      <c r="I26" s="58"/>
+      <c r="J26" s="58"/>
+      <c r="K26" s="59"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="63"/>
+      <c r="B27" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="D27" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="E27" s="64"/>
+      <c r="F27" s="64"/>
+      <c r="G27" s="64"/>
+      <c r="H27" s="64"/>
+      <c r="I27" s="64"/>
+      <c r="J27" s="64"/>
+      <c r="K27" s="61"/>
+    </row>
+    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="63"/>
+      <c r="B28" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="52"/>
+      <c r="D28" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" s="61"/>
+      <c r="F28" s="60" t="s">
+        <v>8</v>
+      </c>
+      <c r="G28" s="61"/>
+      <c r="H28" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="61"/>
+      <c r="J28" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="F22" s="16" t="str">
-        <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="G22" s="16" t="str">
-        <f>IF(F22="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H22" s="16" t="str">
-        <f t="shared" si="16"/>
-        <v/>
-      </c>
-      <c r="I22" s="16" t="str">
-        <f>IF(H22="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="16" t="str">
-        <f t="shared" si="18"/>
-        <v/>
-      </c>
-      <c r="K22" s="16" t="str">
-        <f t="shared" si="19"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="61"/>
-      <c r="B23" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="37">
-        <f>E23+G23+I23+K23</f>
-        <v>70</v>
-      </c>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19">
-        <f>SUM(E13:E22)</f>
-        <v>70</v>
-      </c>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19">
-        <f>SUM(G13:G22)</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19">
-        <f>SUM(I13:I22)</f>
-        <v>0</v>
-      </c>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19">
-        <f>SUM(K13:K22)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="50"/>
-      <c r="B24" s="36" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" s="20">
-        <f>VLOOKUP(C23,ESCALA_IEP!A2:B142,2,FALSE)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="C27" s="52">
-        <f>$B$4</f>
-        <v>0</v>
-      </c>
-      <c r="D27" s="53"/>
-      <c r="E27" s="53"/>
-      <c r="F27" s="53"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="53"/>
-      <c r="I27" s="53"/>
-      <c r="J27" s="53"/>
-      <c r="K27" s="54"/>
-    </row>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="61"/>
-      <c r="B28" s="50"/>
-      <c r="C28" s="55"/>
-      <c r="D28" s="56"/>
-      <c r="E28" s="56"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="56"/>
-      <c r="H28" s="56"/>
-      <c r="I28" s="56"/>
-      <c r="J28" s="56"/>
-      <c r="K28" s="57"/>
-    </row>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="61"/>
-      <c r="B29" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="51" t="s">
-        <v>4</v>
-      </c>
-      <c r="D29" s="58" t="s">
-        <v>5</v>
-      </c>
-      <c r="E29" s="62"/>
-      <c r="F29" s="62"/>
-      <c r="G29" s="62"/>
-      <c r="H29" s="62"/>
-      <c r="I29" s="62"/>
-      <c r="J29" s="62"/>
-      <c r="K29" s="59"/>
-    </row>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="61"/>
-      <c r="B30" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="50"/>
-      <c r="D30" s="58" t="s">
-        <v>7</v>
-      </c>
-      <c r="E30" s="59"/>
-      <c r="F30" s="58" t="s">
-        <v>8</v>
-      </c>
-      <c r="G30" s="59"/>
-      <c r="H30" s="58" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" s="59"/>
-      <c r="J30" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="K30" s="59"/>
-    </row>
-    <row r="31" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="61"/>
-      <c r="B31" s="35" t="str">
+      <c r="K28" s="61"/>
+    </row>
+    <row r="29" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="63"/>
+      <c r="B29" s="35" t="str">
         <f>RUBRICA!A7</f>
         <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
       </c>
+      <c r="C29" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E29" s="16">
+        <f>IF(D29="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="G29" s="16" t="str">
+        <f>IF(F29="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H29" s="16" t="str">
+        <f t="shared" ref="H29:H30" si="21">IF($C29=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I29" s="16" t="str">
+        <f>IF(H29="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="16" t="str">
+        <f t="shared" ref="J29:J30" si="22">IF($C29=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K29" s="16" t="str">
+        <f t="shared" ref="K29:K30" si="23">IF($J29="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="63"/>
+      <c r="B30" s="35" t="str">
+        <f>RUBRICA!A15</f>
+        <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
+      </c>
+      <c r="C30" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D30" s="16" t="str">
+        <f t="shared" ref="D30" si="24">IF($C30=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E30" s="16">
+        <f>IF(D30="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F30" s="16" t="str">
+        <f t="shared" ref="F30" si="25">IF($C30=L,"X","")</f>
+        <v/>
+      </c>
+      <c r="G30" s="16" t="str">
+        <f>IF(F30="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H30" s="16" t="str">
+        <f t="shared" si="21"/>
+        <v/>
+      </c>
+      <c r="I30" s="16" t="str">
+        <f>IF(H30="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="16" t="str">
+        <f t="shared" si="22"/>
+        <v/>
+      </c>
+      <c r="K30" s="16" t="str">
+        <f t="shared" si="23"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="63"/>
+      <c r="B31" s="35" t="str">
+        <f>RUBRICA!A17</f>
+        <v>13. Colaboración y trabajo en equipo *</v>
+      </c>
       <c r="C31" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D31" s="16" t="str">
-        <f t="shared" ref="D31:D32" si="25">IF($C31=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E31" s="16">
+      <c r="D31" s="16" t="s">
+        <v>96</v>
+      </c>
+      <c r="E31" s="16" t="str">
         <f>IF(D31="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F31" s="16" t="str">
-        <f t="shared" ref="F31:F32" si="26">IF($C31=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G31" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F31" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="G31" s="16">
         <f>IF(F31="X",60*0.1,"")</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="H31" s="16" t="str">
-        <f t="shared" ref="H31:H32" si="27">IF($C31=ML,"X","")</f>
+        <f>IF($C31=ML,"X","")</f>
         <v/>
       </c>
       <c r="I31" s="16" t="str">
@@ -2148,233 +2199,233 @@
         <v/>
       </c>
       <c r="J31" s="16" t="str">
-        <f t="shared" ref="J31:J32" si="28">IF($C31=NL,"X","")</f>
+        <f>IF($C31=NL,"X","")</f>
         <v/>
       </c>
       <c r="K31" s="16" t="str">
-        <f t="shared" ref="K31:K32" si="29">IF($J31="X",0,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="61"/>
-      <c r="B32" s="35" t="str">
+        <f>IF($J31="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="63"/>
+      <c r="B32" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="18">
+        <f>E32+G32+I32+K32</f>
+        <v>26</v>
+      </c>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19">
+        <f>SUM(E29:E31)</f>
+        <v>20</v>
+      </c>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19">
+        <f t="shared" ref="G32:K32" si="26">SUM(G29:G31)</f>
+        <v>6</v>
+      </c>
+      <c r="H32" s="19"/>
+      <c r="I32" s="19">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+      <c r="J32" s="19"/>
+      <c r="K32" s="19">
+        <f t="shared" si="26"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="52"/>
+      <c r="B33" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="20">
+        <f>VLOOKUP(C32,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="22"/>
+      <c r="C34" s="23"/>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="22"/>
+      <c r="C35" s="23"/>
+    </row>
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="54" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="D37" s="55"/>
+      <c r="E37" s="55"/>
+      <c r="F37" s="55"/>
+      <c r="G37" s="55"/>
+      <c r="H37" s="55"/>
+      <c r="I37" s="55"/>
+      <c r="J37" s="55"/>
+      <c r="K37" s="56"/>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="63"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="57"/>
+      <c r="D38" s="58"/>
+      <c r="E38" s="58"/>
+      <c r="F38" s="58"/>
+      <c r="G38" s="58"/>
+      <c r="H38" s="58"/>
+      <c r="I38" s="58"/>
+      <c r="J38" s="58"/>
+      <c r="K38" s="59"/>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="63"/>
+      <c r="B39" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="D39" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="E39" s="64"/>
+      <c r="F39" s="64"/>
+      <c r="G39" s="64"/>
+      <c r="H39" s="64"/>
+      <c r="I39" s="64"/>
+      <c r="J39" s="64"/>
+      <c r="K39" s="61"/>
+    </row>
+    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="63"/>
+      <c r="B40" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="52"/>
+      <c r="D40" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="E40" s="61"/>
+      <c r="F40" s="60" t="s">
+        <v>8</v>
+      </c>
+      <c r="G40" s="61"/>
+      <c r="H40" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="I40" s="61"/>
+      <c r="J40" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="K40" s="61"/>
+    </row>
+    <row r="41" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="63"/>
+      <c r="B41" s="35" t="str">
+        <f>RUBRICA!A7</f>
+        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
+      </c>
+      <c r="C41" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="16" t="str">
+        <f t="shared" ref="D41:D42" si="27">IF($C41=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E41" s="16">
+        <f>IF(D41="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F41" s="16" t="str">
+        <f t="shared" ref="F41:F42" si="28">IF($C41=L,"X","")</f>
+        <v/>
+      </c>
+      <c r="G41" s="16" t="str">
+        <f>IF(F41="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H41" s="16" t="str">
+        <f t="shared" ref="H41:H42" si="29">IF($C41=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I41" s="16" t="str">
+        <f>IF(H41="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J41" s="16" t="str">
+        <f t="shared" ref="J41:J42" si="30">IF($C41=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K41" s="16" t="str">
+        <f t="shared" ref="K41:K42" si="31">IF($J41="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="24" x14ac:dyDescent="0.25">
+      <c r="A42" s="63"/>
+      <c r="B42" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
       </c>
-      <c r="C32" s="33" t="s">
+      <c r="C42" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D32" s="16" t="str">
-        <f t="shared" si="25"/>
+      <c r="D42" s="16" t="str">
+        <f t="shared" si="27"/>
         <v>X</v>
       </c>
-      <c r="E32" s="16">
-        <f>IF(D32="X",100*0.1,"")</f>
+      <c r="E42" s="16">
+        <f>IF(D42="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F32" s="16" t="str">
-        <f t="shared" si="26"/>
-        <v/>
-      </c>
-      <c r="G32" s="16" t="str">
-        <f>IF(F32="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H32" s="16" t="str">
-        <f t="shared" si="27"/>
-        <v/>
-      </c>
-      <c r="I32" s="16" t="str">
-        <f>IF(H32="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="16" t="str">
+      <c r="F42" s="16" t="str">
         <f t="shared" si="28"/>
         <v/>
       </c>
-      <c r="K32" s="16" t="str">
+      <c r="G42" s="16" t="str">
+        <f>IF(F42="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H42" s="16" t="str">
         <f t="shared" si="29"/>
         <v/>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="61"/>
-      <c r="B33" s="35" t="str">
+      <c r="I42" s="16" t="str">
+        <f>IF(H42="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J42" s="16" t="str">
+        <f t="shared" si="30"/>
+        <v/>
+      </c>
+      <c r="K42" s="16" t="str">
+        <f t="shared" si="31"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="63"/>
+      <c r="B43" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
       </c>
-      <c r="C33" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="16" t="str">
-        <f>IF($C33=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E33" s="16">
-        <f>IF(D33="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F33" s="16" t="str">
-        <f>IF($C33=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G33" s="16" t="str">
-        <f>IF(F33="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H33" s="16" t="str">
-        <f>IF($C33=ML,"X","")</f>
-        <v/>
-      </c>
-      <c r="I33" s="16" t="str">
-        <f>IF(H33="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="16" t="str">
-        <f>IF($C33=NL,"X","")</f>
-        <v/>
-      </c>
-      <c r="K33" s="16" t="str">
-        <f>IF($J33="X",0,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="61"/>
-      <c r="B34" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C34" s="18">
-        <f>E34+G34+I34+K34</f>
-        <v>30</v>
-      </c>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19">
-        <f>SUM(E31:E33)</f>
-        <v>30</v>
-      </c>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19">
-        <f t="shared" ref="G34:K34" si="30">SUM(G31:G33)</f>
-        <v>0</v>
-      </c>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19">
-        <f t="shared" si="30"/>
-        <v>0</v>
-      </c>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19">
-        <f t="shared" si="30"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="50"/>
-      <c r="B35" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" s="20">
-        <f>VLOOKUP(C34,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="22"/>
-      <c r="C36" s="23"/>
-    </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="22"/>
-      <c r="C37" s="23"/>
-    </row>
-    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="B39" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="C39" s="52">
-        <f>B5</f>
-        <v>0</v>
-      </c>
-      <c r="D39" s="53"/>
-      <c r="E39" s="53"/>
-      <c r="F39" s="53"/>
-      <c r="G39" s="53"/>
-      <c r="H39" s="53"/>
-      <c r="I39" s="53"/>
-      <c r="J39" s="53"/>
-      <c r="K39" s="54"/>
-    </row>
-    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="61"/>
-      <c r="B40" s="50"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="56"/>
-      <c r="E40" s="56"/>
-      <c r="F40" s="56"/>
-      <c r="G40" s="56"/>
-      <c r="H40" s="56"/>
-      <c r="I40" s="56"/>
-      <c r="J40" s="56"/>
-      <c r="K40" s="57"/>
-    </row>
-    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="61"/>
-      <c r="B41" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C41" s="51" t="s">
-        <v>4</v>
-      </c>
-      <c r="D41" s="58" t="s">
-        <v>5</v>
-      </c>
-      <c r="E41" s="62"/>
-      <c r="F41" s="62"/>
-      <c r="G41" s="62"/>
-      <c r="H41" s="62"/>
-      <c r="I41" s="62"/>
-      <c r="J41" s="62"/>
-      <c r="K41" s="59"/>
-    </row>
-    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="61"/>
-      <c r="B42" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C42" s="50"/>
-      <c r="D42" s="58" t="s">
-        <v>7</v>
-      </c>
-      <c r="E42" s="59"/>
-      <c r="F42" s="58" t="s">
-        <v>8</v>
-      </c>
-      <c r="G42" s="59"/>
-      <c r="H42" s="58" t="s">
-        <v>16</v>
-      </c>
-      <c r="I42" s="59"/>
-      <c r="J42" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="K42" s="59"/>
-    </row>
-    <row r="43" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="61"/>
-      <c r="B43" s="35" t="str">
-        <f>RUBRICA!A7</f>
-        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
-      </c>
       <c r="C43" s="33" t="s">
         <v>7</v>
       </c>
       <c r="D43" s="16" t="str">
-        <f t="shared" ref="D43:D44" si="31">IF($C43=CL,"X","")</f>
+        <f>IF($C43=CL,"X","")</f>
         <v>X</v>
       </c>
       <c r="E43" s="16">
@@ -2382,7 +2433,7 @@
         <v>10</v>
       </c>
       <c r="F43" s="16" t="str">
-        <f t="shared" ref="F43:F44" si="32">IF($C43=L,"X","")</f>
+        <f>IF($C43=L,"X","")</f>
         <v/>
       </c>
       <c r="G43" s="16" t="str">
@@ -2390,7 +2441,7 @@
         <v/>
       </c>
       <c r="H43" s="16" t="str">
-        <f t="shared" ref="H43:H44" si="33">IF($C43=ML,"X","")</f>
+        <f>IF($C43=ML,"X","")</f>
         <v/>
       </c>
       <c r="I43" s="16" t="str">
@@ -2398,232 +2449,232 @@
         <v/>
       </c>
       <c r="J43" s="16" t="str">
-        <f t="shared" ref="J43:J44" si="34">IF($C43=NL,"X","")</f>
+        <f>IF($C43=NL,"X","")</f>
         <v/>
       </c>
       <c r="K43" s="16" t="str">
-        <f t="shared" ref="K43:K44" si="35">IF($J43="X",0,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="24" x14ac:dyDescent="0.25">
-      <c r="A44" s="61"/>
-      <c r="B44" s="35" t="str">
+        <f>IF($J43="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="63"/>
+      <c r="B44" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="18">
+        <f>E44+G44+I44+K44</f>
+        <v>30</v>
+      </c>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19">
+        <f>SUM(E41:E43)</f>
+        <v>30</v>
+      </c>
+      <c r="F44" s="19"/>
+      <c r="G44" s="19">
+        <f t="shared" ref="G44" si="32">SUM(G41:G43)</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="19"/>
+      <c r="I44" s="19">
+        <f t="shared" ref="I44" si="33">SUM(I41:I43)</f>
+        <v>0</v>
+      </c>
+      <c r="J44" s="19"/>
+      <c r="K44" s="19">
+        <f t="shared" ref="K44" si="34">SUM(K41:K43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="52"/>
+      <c r="B45" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="20">
+        <f>VLOOKUP(C44,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="22"/>
+      <c r="C46" s="23"/>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="22"/>
+      <c r="C47" s="23"/>
+    </row>
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" s="51" t="s">
+        <v>14</v>
+      </c>
+      <c r="C48" s="54" t="e">
+        <f>#REF!</f>
+        <v>#REF!</v>
+      </c>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="55"/>
+      <c r="J48" s="55"/>
+      <c r="K48" s="56"/>
+    </row>
+    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="63"/>
+      <c r="B49" s="52"/>
+      <c r="C49" s="57"/>
+      <c r="D49" s="58"/>
+      <c r="E49" s="58"/>
+      <c r="F49" s="58"/>
+      <c r="G49" s="58"/>
+      <c r="H49" s="58"/>
+      <c r="I49" s="58"/>
+      <c r="J49" s="58"/>
+      <c r="K49" s="59"/>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="63"/>
+      <c r="B50" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C50" s="53" t="s">
+        <v>4</v>
+      </c>
+      <c r="D50" s="60" t="s">
+        <v>5</v>
+      </c>
+      <c r="E50" s="64"/>
+      <c r="F50" s="64"/>
+      <c r="G50" s="64"/>
+      <c r="H50" s="64"/>
+      <c r="I50" s="64"/>
+      <c r="J50" s="64"/>
+      <c r="K50" s="61"/>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="63"/>
+      <c r="B51" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="52"/>
+      <c r="D51" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" s="61"/>
+      <c r="F51" s="60" t="s">
+        <v>8</v>
+      </c>
+      <c r="G51" s="61"/>
+      <c r="H51" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" s="61"/>
+      <c r="J51" s="60" t="s">
+        <v>10</v>
+      </c>
+      <c r="K51" s="61"/>
+    </row>
+    <row r="52" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="63"/>
+      <c r="B52" s="35" t="str">
+        <f>RUBRICA!A7</f>
+        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
+      </c>
+      <c r="C52" s="33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D52" s="16" t="str">
+        <f t="shared" ref="D52:D53" si="35">IF($C52=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E52" s="16">
+        <f>IF(D52="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F52" s="16" t="str">
+        <f t="shared" ref="F52:F53" si="36">IF($C52=L,"X","")</f>
+        <v/>
+      </c>
+      <c r="G52" s="16" t="str">
+        <f>IF(F52="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H52" s="16" t="str">
+        <f t="shared" ref="H52:H53" si="37">IF($C52=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I52" s="16" t="str">
+        <f>IF(H52="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J52" s="16" t="str">
+        <f t="shared" ref="J52:J53" si="38">IF($C52=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K52" s="16" t="str">
+        <f t="shared" ref="K52:K53" si="39">IF($J52="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="24" x14ac:dyDescent="0.25">
+      <c r="A53" s="63"/>
+      <c r="B53" s="35" t="str">
         <f>RUBRICA!A15</f>
         <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
       </c>
-      <c r="C44" s="33" t="s">
+      <c r="C53" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D44" s="16" t="str">
-        <f t="shared" si="31"/>
+      <c r="D53" s="16" t="str">
+        <f t="shared" si="35"/>
         <v>X</v>
       </c>
-      <c r="E44" s="16">
-        <f>IF(D44="X",100*0.1,"")</f>
+      <c r="E53" s="16">
+        <f>IF(D53="X",100*0.1,"")</f>
         <v>10</v>
       </c>
-      <c r="F44" s="16" t="str">
-        <f t="shared" si="32"/>
-        <v/>
-      </c>
-      <c r="G44" s="16" t="str">
-        <f>IF(F44="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H44" s="16" t="str">
-        <f t="shared" si="33"/>
-        <v/>
-      </c>
-      <c r="I44" s="16" t="str">
-        <f>IF(H44="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J44" s="16" t="str">
-        <f t="shared" si="34"/>
-        <v/>
-      </c>
-      <c r="K44" s="16" t="str">
-        <f t="shared" si="35"/>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="61"/>
-      <c r="B45" s="35" t="str">
+      <c r="F53" s="16" t="str">
+        <f t="shared" si="36"/>
+        <v/>
+      </c>
+      <c r="G53" s="16" t="str">
+        <f>IF(F53="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H53" s="16" t="str">
+        <f t="shared" si="37"/>
+        <v/>
+      </c>
+      <c r="I53" s="16" t="str">
+        <f>IF(H53="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J53" s="16" t="str">
+        <f t="shared" si="38"/>
+        <v/>
+      </c>
+      <c r="K53" s="16" t="str">
+        <f t="shared" si="39"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="63"/>
+      <c r="B54" s="35" t="str">
         <f>RUBRICA!A17</f>
         <v>13. Colaboración y trabajo en equipo *</v>
       </c>
-      <c r="C45" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D45" s="16" t="str">
-        <f>IF($C45=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E45" s="16">
-        <f>IF(D45="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F45" s="16" t="str">
-        <f>IF($C45=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G45" s="16" t="str">
-        <f>IF(F45="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H45" s="16" t="str">
-        <f>IF($C45=ML,"X","")</f>
-        <v/>
-      </c>
-      <c r="I45" s="16" t="str">
-        <f>IF(H45="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J45" s="16" t="str">
-        <f>IF($C45=NL,"X","")</f>
-        <v/>
-      </c>
-      <c r="K45" s="16" t="str">
-        <f>IF($J45="X",0,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="61"/>
-      <c r="B46" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C46" s="18">
-        <f>E46+G46+I46+K46</f>
-        <v>30</v>
-      </c>
-      <c r="D46" s="19"/>
-      <c r="E46" s="19">
-        <f>SUM(E43:E45)</f>
-        <v>30</v>
-      </c>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19">
-        <f t="shared" ref="G46" si="36">SUM(G43:G45)</f>
-        <v>0</v>
-      </c>
-      <c r="H46" s="19"/>
-      <c r="I46" s="19">
-        <f t="shared" ref="I46" si="37">SUM(I43:I45)</f>
-        <v>0</v>
-      </c>
-      <c r="J46" s="19"/>
-      <c r="K46" s="19">
-        <f t="shared" ref="K46" si="38">SUM(K43:K45)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="50"/>
-      <c r="B47" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C47" s="20">
-        <f>VLOOKUP(C46,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="22"/>
-      <c r="C48" s="23"/>
-    </row>
-    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="22"/>
-      <c r="C49" s="23"/>
-    </row>
-    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="B50" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="C50" s="52">
-        <f>B6</f>
-        <v>0</v>
-      </c>
-      <c r="D50" s="53"/>
-      <c r="E50" s="53"/>
-      <c r="F50" s="53"/>
-      <c r="G50" s="53"/>
-      <c r="H50" s="53"/>
-      <c r="I50" s="53"/>
-      <c r="J50" s="53"/>
-      <c r="K50" s="54"/>
-    </row>
-    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="61"/>
-      <c r="B51" s="50"/>
-      <c r="C51" s="55"/>
-      <c r="D51" s="56"/>
-      <c r="E51" s="56"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="56"/>
-      <c r="H51" s="56"/>
-      <c r="I51" s="56"/>
-      <c r="J51" s="56"/>
-      <c r="K51" s="57"/>
-    </row>
-    <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="61"/>
-      <c r="B52" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C52" s="51" t="s">
-        <v>4</v>
-      </c>
-      <c r="D52" s="58" t="s">
-        <v>5</v>
-      </c>
-      <c r="E52" s="62"/>
-      <c r="F52" s="62"/>
-      <c r="G52" s="62"/>
-      <c r="H52" s="62"/>
-      <c r="I52" s="62"/>
-      <c r="J52" s="62"/>
-      <c r="K52" s="59"/>
-    </row>
-    <row r="53" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="61"/>
-      <c r="B53" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C53" s="50"/>
-      <c r="D53" s="58" t="s">
-        <v>7</v>
-      </c>
-      <c r="E53" s="59"/>
-      <c r="F53" s="58" t="s">
-        <v>8</v>
-      </c>
-      <c r="G53" s="59"/>
-      <c r="H53" s="58" t="s">
-        <v>16</v>
-      </c>
-      <c r="I53" s="59"/>
-      <c r="J53" s="58" t="s">
-        <v>10</v>
-      </c>
-      <c r="K53" s="59"/>
-    </row>
-    <row r="54" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="61"/>
-      <c r="B54" s="35" t="str">
-        <f>RUBRICA!A7</f>
-        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
-      </c>
       <c r="C54" s="33" t="s">
         <v>7</v>
       </c>
       <c r="D54" s="16" t="str">
-        <f t="shared" ref="D54:D55" si="39">IF($C54=CL,"X","")</f>
+        <f>IF($C54=CL,"X","")</f>
         <v>X</v>
       </c>
       <c r="E54" s="16">
@@ -2631,7 +2682,7 @@
         <v>10</v>
       </c>
       <c r="F54" s="16" t="str">
-        <f t="shared" ref="F54:F55" si="40">IF($C54=L,"X","")</f>
+        <f>IF($C54=L,"X","")</f>
         <v/>
       </c>
       <c r="G54" s="16" t="str">
@@ -2639,7 +2690,7 @@
         <v/>
       </c>
       <c r="H54" s="16" t="str">
-        <f t="shared" ref="H54:H55" si="41">IF($C54=ML,"X","")</f>
+        <f>IF($C54=ML,"X","")</f>
         <v/>
       </c>
       <c r="I54" s="16" t="str">
@@ -2647,154 +2698,72 @@
         <v/>
       </c>
       <c r="J54" s="16" t="str">
-        <f t="shared" ref="J54:J55" si="42">IF($C54=NL,"X","")</f>
+        <f>IF($C54=NL,"X","")</f>
         <v/>
       </c>
       <c r="K54" s="16" t="str">
-        <f t="shared" ref="K54:K55" si="43">IF($J54="X",0,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="24" x14ac:dyDescent="0.25">
-      <c r="A55" s="61"/>
-      <c r="B55" s="35" t="str">
-        <f>RUBRICA!A15</f>
-        <v>11. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
-      </c>
-      <c r="C55" s="33" t="s">
+        <f>IF($J54="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="63"/>
+      <c r="B55" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="C55" s="18">
+        <f>E55+G55+I55+K55</f>
+        <v>30</v>
+      </c>
+      <c r="D55" s="19">
+        <f>COUNTIF(D53:D54,"X")</f>
+        <v>2</v>
+      </c>
+      <c r="E55" s="19">
+        <f>SUM(E52:E54)</f>
+        <v>30</v>
+      </c>
+      <c r="F55" s="19">
+        <f t="shared" ref="F55" si="40">SUM(F52:F54)</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="19">
+        <f t="shared" ref="G55" si="41">SUM(G52:G54)</f>
+        <v>0</v>
+      </c>
+      <c r="H55" s="19">
+        <f t="shared" ref="H55" si="42">SUM(H52:H54)</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="19">
+        <f t="shared" ref="I55" si="43">SUM(I52:I54)</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="19">
+        <f t="shared" ref="J55" si="44">SUM(J52:J54)</f>
+        <v>0</v>
+      </c>
+      <c r="K55" s="19">
+        <f t="shared" ref="K55" si="45">SUM(K52:K54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="52"/>
+      <c r="B56" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C56" s="20">
+        <f>VLOOKUP(C55,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
         <v>7</v>
       </c>
-      <c r="D55" s="16" t="str">
-        <f t="shared" si="39"/>
-        <v>X</v>
-      </c>
-      <c r="E55" s="16">
-        <f>IF(D55="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F55" s="16" t="str">
-        <f t="shared" si="40"/>
-        <v/>
-      </c>
-      <c r="G55" s="16" t="str">
-        <f>IF(F55="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H55" s="16" t="str">
-        <f t="shared" si="41"/>
-        <v/>
-      </c>
-      <c r="I55" s="16" t="str">
-        <f>IF(H55="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J55" s="16" t="str">
-        <f t="shared" si="42"/>
-        <v/>
-      </c>
-      <c r="K55" s="16" t="str">
-        <f t="shared" si="43"/>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="61"/>
-      <c r="B56" s="35" t="str">
-        <f>RUBRICA!A17</f>
-        <v>13. Colaboración y trabajo en equipo *</v>
-      </c>
-      <c r="C56" s="33" t="s">
-        <v>7</v>
-      </c>
-      <c r="D56" s="16" t="str">
-        <f>IF($C56=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E56" s="16">
-        <f>IF(D56="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F56" s="16" t="str">
-        <f>IF($C56=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G56" s="16" t="str">
-        <f>IF(F56="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H56" s="16" t="str">
-        <f>IF($C56=ML,"X","")</f>
-        <v/>
-      </c>
-      <c r="I56" s="16" t="str">
-        <f>IF(H56="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J56" s="16" t="str">
-        <f>IF($C56=NL,"X","")</f>
-        <v/>
-      </c>
-      <c r="K56" s="16" t="str">
-        <f>IF($J56="X",0,"")</f>
-        <v/>
-      </c>
     </row>
     <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="61"/>
-      <c r="B57" s="21" t="s">
-        <v>17</v>
-      </c>
-      <c r="C57" s="18">
-        <f>E57+G57+I57+K57</f>
-        <v>30</v>
-      </c>
-      <c r="D57" s="19">
-        <f>COUNTIF(D55:D56,"X")</f>
-        <v>2</v>
-      </c>
-      <c r="E57" s="19">
-        <f>SUM(E54:E56)</f>
-        <v>30</v>
-      </c>
-      <c r="F57" s="19">
-        <f t="shared" ref="F57" si="44">SUM(F54:F56)</f>
-        <v>0</v>
-      </c>
-      <c r="G57" s="19">
-        <f t="shared" ref="G57" si="45">SUM(G54:G56)</f>
-        <v>0</v>
-      </c>
-      <c r="H57" s="19">
-        <f t="shared" ref="H57" si="46">SUM(H54:H56)</f>
-        <v>0</v>
-      </c>
-      <c r="I57" s="19">
-        <f t="shared" ref="I57" si="47">SUM(I54:I56)</f>
-        <v>0</v>
-      </c>
-      <c r="J57" s="19">
-        <f t="shared" ref="J57" si="48">SUM(J54:J56)</f>
-        <v>0</v>
-      </c>
-      <c r="K57" s="19">
-        <f t="shared" ref="K57" si="49">SUM(K54:K56)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="50"/>
-      <c r="B58" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="C58" s="20">
-        <f>VLOOKUP(C57,ESCALA_TRAB_EQUIP!A2:B62,2,FALSE)</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="22"/>
-      <c r="C59" s="23"/>
-    </row>
+      <c r="B57" s="22"/>
+      <c r="C57" s="23"/>
+    </row>
+    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3663,47 +3632,45 @@
     <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C39:K40"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:K41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="A39:A47"/>
-    <mergeCell ref="A27:A35"/>
+    <mergeCell ref="B37:B38"/>
+    <mergeCell ref="C37:K38"/>
+    <mergeCell ref="C39:C40"/>
+    <mergeCell ref="D39:K39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="A37:A45"/>
+    <mergeCell ref="A25:A33"/>
     <mergeCell ref="E2:E3"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D11:K11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="A11:A24"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:K28"/>
-    <mergeCell ref="C29:C30"/>
-    <mergeCell ref="D29:K29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="D52:K52"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C52:C53"/>
-    <mergeCell ref="C50:K51"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A50:A58"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D9:K9"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="A9:A22"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:K26"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:K27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="D50:K50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="C48:K49"/>
+    <mergeCell ref="J51:K51"/>
+    <mergeCell ref="A48:A56"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4:E6">
+  <conditionalFormatting sqref="C4:E4">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>4</formula>
     </cfRule>
@@ -3712,7 +3679,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Error de Ingreso - Nota debe estar entre 1,0 y 7,0" sqref="C4:E6" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Error de Ingreso - Nota debe estar entre 1,0 y 7,0" sqref="C4:E4" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>1</formula1>
       <formula2>7</formula2>
     </dataValidation>
@@ -3726,7 +3693,7 @@
           <x14:formula1>
             <xm:f>'RELEVANCIA-PUNTAJE'!$B$2:$E$2</xm:f>
           </x14:formula1>
-          <xm:sqref>C13:C22 C54:C56 C43:C45 C31:C33</xm:sqref>
+          <xm:sqref>C11:C20 C52:C54 C41:C43 C29:C31</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3748,25 +3715,25 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="71" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="72" t="s">
+      <c r="B2" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="69" t="s">
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="71" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="70"/>
-      <c r="B3" s="75" t="s">
+      <c r="A3" s="72"/>
+      <c r="B3" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="75" t="s">
+      <c r="C3" s="77" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="25" t="s">
@@ -3775,19 +3742,19 @@
       <c r="E3" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="70"/>
+      <c r="F3" s="72"/>
     </row>
     <row r="4" spans="1:6" ht="57.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="71"/>
-      <c r="B4" s="76"/>
-      <c r="C4" s="76"/>
+      <c r="A4" s="73"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
       <c r="D4" s="26">
         <v>-0.3</v>
       </c>
       <c r="E4" s="26">
         <v>0</v>
       </c>
-      <c r="F4" s="71"/>
+      <c r="F4" s="73"/>
     </row>
     <row r="5" spans="1:6" ht="77.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="38" t="s">
@@ -4050,13 +4017,13 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="66" t="s">
+      <c r="A18" s="68" t="s">
         <v>89</v>
       </c>
-      <c r="B18" s="67"/>
-      <c r="C18" s="67"/>
-      <c r="D18" s="67"/>
-      <c r="E18" s="68"/>
+      <c r="B18" s="69"/>
+      <c r="C18" s="69"/>
+      <c r="D18" s="69"/>
+      <c r="E18" s="70"/>
       <c r="F18" s="29">
         <v>1</v>
       </c>
@@ -8931,7 +8898,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="79" t="s">
         <v>92</v>
       </c>
       <c r="B1" s="7" t="s">
@@ -8942,7 +8909,7 @@
       <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="78"/>
+      <c r="A2" s="80"/>
       <c r="B2" s="10" t="s">
         <v>7</v>
       </c>

</xml_diff>